<commit_message>
Updated Models and Monitors
</commit_message>
<xml_diff>
--- a/financial_models/Bank_Monitor.xlsx
+++ b/financial_models/Bank_Monitor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerry\PycharmProjects\Invest_Proc\financial_models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7770292-F970-4AA4-8488-3B55C8DAB788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0FF9D08-A2B1-44E9-AA16-CAAAB78307D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6150" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,6 +22,8 @@
     <definedName name="Benchmark_yield">Assumptions!$C$8</definedName>
     <definedName name="Entry_yield">Assumptions!$C$7</definedName>
     <definedName name="g">Assumptions!$C$4</definedName>
+    <definedName name="HKDCNY">Assumptions!$C$13</definedName>
+    <definedName name="HKDUSD">Assumptions!$C$12</definedName>
     <definedName name="Holding_Period">Assumptions!$C$5</definedName>
     <definedName name="k">Assumptions!$C$3</definedName>
     <definedName name="Target_return">Assumptions!$C$6</definedName>
@@ -33,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="132">
   <si>
     <t>Name</t>
   </si>
@@ -110,9 +112,6 @@
     <t>公司名称</t>
   </si>
   <si>
-    <t>每股净资产</t>
-  </si>
-  <si>
     <t>HK:1398 / SH:601398</t>
   </si>
   <si>
@@ -132,9 +131,6 @@
   </si>
   <si>
     <t>Trading Currency</t>
-  </si>
-  <si>
-    <t>listed in China</t>
   </si>
   <si>
     <t>YYYY-MM-DD</t>
@@ -150,9 +146,6 @@
 per share</t>
   </si>
   <si>
-    <t>From last Financial year</t>
-  </si>
-  <si>
     <t>派息率</t>
   </si>
   <si>
@@ -171,9 +164,6 @@
     <t>Tangible Common Equity per Share</t>
   </si>
   <si>
-    <t>Common Equity per share</t>
-  </si>
-  <si>
     <t>ROTCE = Core Net income ÷ Tangible common equity (goodwill &amp; intangibles stripped out).</t>
   </si>
   <si>
@@ -183,9 +173,6 @@
     <t>ROTCE</t>
   </si>
   <si>
-    <t>Total Assets/Total Equity</t>
-  </si>
-  <si>
     <t>DuPont for ROTCE</t>
   </si>
   <si>
@@ -237,12 +224,6 @@
     <t>Company Info.</t>
   </si>
   <si>
-    <t>Per Share Metrics</t>
-  </si>
-  <si>
-    <t>上一个财年EPS</t>
-  </si>
-  <si>
     <t>上一个财年核心EPS</t>
   </si>
   <si>
@@ -262,9 +243,6 @@
   </si>
   <si>
     <t>Valuation</t>
-  </si>
-  <si>
-    <t>隐含公允市净率</t>
   </si>
   <si>
     <t>隐含公允股价</t>
@@ -369,34 +347,18 @@
     <t>Last FY Core shareholders' EPS</t>
   </si>
   <si>
-    <t>Last FY 
-shareholders' EPS</t>
-  </si>
-  <si>
     <t>有形净资产</t>
   </si>
   <si>
     <t>核心净利润</t>
   </si>
   <si>
-    <t>Last FY Core shareholders' Net Income</t>
-  </si>
-  <si>
     <t>收入</t>
   </si>
   <si>
-    <t>Revenue</t>
-  </si>
-  <si>
-    <t>Total Assets</t>
-  </si>
-  <si>
     <t>总资产</t>
   </si>
   <si>
-    <t>Tangible Common Equity (TBV)</t>
-  </si>
-  <si>
     <t>CET1</t>
   </si>
   <si>
@@ -409,18 +371,80 @@
     <t>Profibilities and Efficiency</t>
   </si>
   <si>
-    <t>Share Outstanding</t>
-  </si>
-  <si>
     <t>股数</t>
+  </si>
+  <si>
+    <t>HSBC</t>
+  </si>
+  <si>
+    <t>HK:0005</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>Total Assets
+(in Millions)</t>
+  </si>
+  <si>
+    <t>Tangible Common Equity (TBV)
+(in Millions)</t>
+  </si>
+  <si>
+    <t>Revenue
+(in Millions)</t>
+  </si>
+  <si>
+    <t>Last FY Core shareholders' Net Income (in Millions)</t>
+  </si>
+  <si>
+    <t>From End Date of Last Statement</t>
+  </si>
+  <si>
+    <t>From the Last Annual Report</t>
+  </si>
+  <si>
+    <t>Listing Symbol</t>
+  </si>
+  <si>
+    <t>Latest</t>
+  </si>
+  <si>
+    <t>Latest Share Outstanding</t>
+  </si>
+  <si>
+    <t>Total Assets/TBV</t>
+  </si>
+  <si>
+    <t>HKD</t>
+  </si>
+  <si>
+    <t>Forex</t>
+  </si>
+  <si>
+    <t>HKDUSD</t>
+  </si>
+  <si>
+    <t>HKDCNY</t>
+  </si>
+  <si>
+    <t>Forex Pair</t>
+  </si>
+  <si>
+    <t>Forex Rate</t>
+  </si>
+  <si>
+    <t>公允市净率倍数</t>
+  </si>
+  <si>
+    <t>From last Financial year (in trading currency)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
-    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00;[Red]\-&quot;$&quot;#,##0.00"/>
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd;@"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="#,##0.000"/>
@@ -651,8 +675,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -681,8 +703,38 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -690,66 +742,38 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -1075,7 +1099,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21D2ED91-59EB-437C-A4C2-C114238F9C2A}">
-  <dimension ref="B2:D24"/>
+  <dimension ref="B2:D30"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.59765625" customWidth="1"/>
@@ -1092,12 +1116,12 @@
         <v>2</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B3" s="1" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C3" s="14">
         <v>0.1</v>
@@ -1106,18 +1130,18 @@
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B4" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C4" s="14">
         <v>0.02</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B5" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C5" s="15">
         <v>3</v>
@@ -1126,7 +1150,7 @@
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B6" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C6" s="14">
         <v>0.29465259038036606</v>
@@ -1135,7 +1159,7 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B7" s="1" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C7" s="14">
         <v>0.20075184365903009</v>
@@ -1144,7 +1168,7 @@
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B8" s="1" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C8" s="14">
         <v>0.1174</v>
@@ -1153,61 +1177,100 @@
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B9" s="1" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="C9" s="14">
         <v>7.2499999999999995E-2</v>
       </c>
       <c r="D9" s="1"/>
     </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B11" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C12" s="52">
+        <v>7.8</v>
+      </c>
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B13" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C13" s="52">
+        <v>0.89</v>
+      </c>
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B14" s="1"/>
+      <c r="C14" s="51"/>
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B15" s="1"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="1"/>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B18" s="17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B13" t="s">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B21" t="s">
         <v>42</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B15" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B16" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B17" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B19" s="20" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B20" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B24" t="s">
-        <v>53</v>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B25" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B28" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B29" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B30" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1218,22 +1281,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC6E8AA2-48F2-4368-B9E3-BA821DC1A767}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B2:AG12"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" outlineLevelCol="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
     <col min="2" max="4" width="18.6640625" customWidth="1"/>
-    <col min="5" max="11" width="18.6640625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="12" max="12" width="18.6640625" customWidth="1" collapsed="1"/>
-    <col min="13" max="18" width="18.6640625" customWidth="1"/>
-    <col min="19" max="24" width="18.6640625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="25" max="25" width="18.796875" customWidth="1" collapsed="1"/>
-    <col min="26" max="33" width="18.796875" customWidth="1"/>
+    <col min="5" max="12" width="18.6640625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="13" max="13" width="18.6640625" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <col min="14" max="19" width="18.6640625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="20" max="20" width="18.6640625" customWidth="1" collapsed="1"/>
+    <col min="21" max="22" width="18.6640625" customWidth="1"/>
+    <col min="23" max="30" width="18.796875" customWidth="1"/>
+    <col min="31" max="32" width="18.796875" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="18.796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:33" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B2" s="2" t="s">
-        <v>33</v>
+        <v>120</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>16</v>
@@ -1242,318 +1310,320 @@
         <v>17</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="O2" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="P2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Q2" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="R2" s="2" t="s">
-        <v>56</v>
+        <v>123</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="T2" s="2"/>
+        <v>51</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="U2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>60</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="Y2" s="16"/>
+      <c r="Z2" s="16"/>
       <c r="AA2" s="16"/>
       <c r="AB2" s="16"/>
-      <c r="AC2" s="16"/>
-      <c r="AD2" s="16"/>
+      <c r="AC2" s="2"/>
+      <c r="AD2" s="2"/>
       <c r="AE2" s="2"/>
       <c r="AF2" s="2"/>
       <c r="AG2" s="2"/>
     </row>
     <row r="3" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="42" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="43"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
+      <c r="I3" s="46"/>
+      <c r="J3" s="46"/>
+      <c r="K3" s="46"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="47" t="s">
+        <v>109</v>
+      </c>
+      <c r="N3" s="47"/>
+      <c r="O3" s="47"/>
+      <c r="P3" s="47"/>
+      <c r="Q3" s="47"/>
+      <c r="R3" s="47"/>
+      <c r="S3" s="48"/>
+      <c r="T3" s="39"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="39"/>
+      <c r="W3" s="40" t="s">
+        <v>68</v>
+      </c>
+      <c r="X3" s="40"/>
+      <c r="Y3" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="Z3" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA3" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="AB3" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC3" s="41" t="s">
+        <v>78</v>
+      </c>
+      <c r="AD3" s="41"/>
+      <c r="AE3" s="41"/>
+      <c r="AF3" s="41"/>
+      <c r="AG3" s="41"/>
+    </row>
+    <row r="4" spans="2:33" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="B4" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="F4" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" s="32" t="s">
+        <v>114</v>
+      </c>
+      <c r="H4" s="32" t="s">
+        <v>115</v>
+      </c>
+      <c r="I4" s="32" t="s">
+        <v>116</v>
+      </c>
+      <c r="J4" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="K4" s="32" t="s">
+        <v>122</v>
+      </c>
+      <c r="L4" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="M4" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="N4" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="O4" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="P4" s="29" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q4" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="R4" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="S4" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="T4" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="U4" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="V4" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="W4" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="X4" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="Y4" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="Z4" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA4" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="AB4" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="AC4" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="AD4" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="AE4" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="AF4" s="21" t="s">
+        <v>129</v>
+      </c>
+      <c r="AG4" s="21" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="2:33" x14ac:dyDescent="0.45">
+      <c r="B5" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" s="33" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" s="33" t="s">
+        <v>105</v>
+      </c>
+      <c r="H5" s="33" t="s">
+        <v>102</v>
+      </c>
+      <c r="I5" s="33" t="s">
+        <v>104</v>
+      </c>
+      <c r="J5" s="33" t="s">
+        <v>103</v>
+      </c>
+      <c r="K5" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="L5" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="M5" s="30" t="s">
+        <v>107</v>
+      </c>
+      <c r="N5" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="O5" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="P5" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q5" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="R5" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="51"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="39" t="s">
-        <v>121</v>
-      </c>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="40"/>
-      <c r="L3" s="35" t="s">
-        <v>122</v>
-      </c>
-      <c r="M3" s="35"/>
-      <c r="N3" s="35"/>
-      <c r="O3" s="35"/>
-      <c r="P3" s="35"/>
-      <c r="Q3" s="35"/>
-      <c r="R3" s="36"/>
-      <c r="S3" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="T3" s="31"/>
-      <c r="U3" s="31"/>
-      <c r="V3" s="31"/>
-      <c r="W3" s="31"/>
-      <c r="X3" s="31"/>
-      <c r="Y3" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="Z3" s="32"/>
-      <c r="AA3" s="33" t="s">
+      <c r="S5" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="T5" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="U5" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="V5" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="W5" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="X5" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="Y5" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="Z5" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA5" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="AB3" s="33" t="s">
+      <c r="AB5" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AC3" s="33" t="s">
-        <v>96</v>
-      </c>
-      <c r="AD3" s="33" t="s">
-        <v>97</v>
-      </c>
-      <c r="AE3" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="AF3" s="34"/>
-      <c r="AG3" s="34"/>
-    </row>
-    <row r="4" spans="2:33" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="B4" s="43" t="s">
-        <v>88</v>
-      </c>
-      <c r="C4" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" s="43" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="41" t="s">
-        <v>82</v>
-      </c>
-      <c r="F4" s="41" t="s">
-        <v>83</v>
-      </c>
-      <c r="G4" s="41" t="s">
-        <v>116</v>
-      </c>
-      <c r="H4" s="41" t="s">
-        <v>118</v>
-      </c>
-      <c r="I4" s="41" t="s">
-        <v>115</v>
-      </c>
-      <c r="J4" s="41" t="s">
-        <v>113</v>
-      </c>
-      <c r="K4" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="L4" s="37" t="s">
-        <v>119</v>
-      </c>
-      <c r="M4" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="N4" s="37" t="s">
-        <v>21</v>
-      </c>
-      <c r="O4" s="37" t="s">
-        <v>48</v>
-      </c>
-      <c r="P4" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q4" s="37" t="s">
-        <v>54</v>
-      </c>
-      <c r="R4" s="37" t="s">
-        <v>71</v>
-      </c>
-      <c r="S4" s="27" t="s">
-        <v>45</v>
-      </c>
-      <c r="T4" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="U4" s="27" t="s">
-        <v>110</v>
-      </c>
-      <c r="V4" s="27" t="s">
-        <v>109</v>
-      </c>
-      <c r="W4" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="X4" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y4" s="25" t="s">
+      <c r="AC5" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="Z4" s="25" t="s">
-        <v>85</v>
-      </c>
-      <c r="AA4" s="21" t="s">
-        <v>105</v>
-      </c>
-      <c r="AB4" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="AC4" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="AD4" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="AE4" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="AF4" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="AG4" s="23" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="5" spans="2:33" x14ac:dyDescent="0.45">
-      <c r="B5" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" s="44" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="E5" s="42" t="s">
-        <v>62</v>
-      </c>
-      <c r="F5" s="42" t="s">
-        <v>61</v>
-      </c>
-      <c r="G5" s="42" t="s">
-        <v>117</v>
-      </c>
-      <c r="H5" s="42" t="s">
-        <v>111</v>
-      </c>
-      <c r="I5" s="42" t="s">
-        <v>114</v>
-      </c>
-      <c r="J5" s="42" t="s">
-        <v>112</v>
-      </c>
-      <c r="K5" s="42" t="s">
-        <v>124</v>
-      </c>
-      <c r="L5" s="38" t="s">
-        <v>120</v>
-      </c>
-      <c r="M5" s="38" t="s">
-        <v>11</v>
-      </c>
-      <c r="N5" s="38" t="s">
-        <v>12</v>
-      </c>
-      <c r="O5" s="38" t="s">
-        <v>74</v>
-      </c>
-      <c r="P5" s="38" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q5" s="38" t="s">
-        <v>73</v>
-      </c>
-      <c r="R5" s="38" t="s">
-        <v>72</v>
-      </c>
-      <c r="S5" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="T5" s="28" t="s">
+      <c r="AD5" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE5" s="22"/>
+      <c r="AF5" s="22"/>
+      <c r="AG5" s="22" t="s">
         <v>70</v>
-      </c>
-      <c r="U5" s="29" t="s">
-        <v>68</v>
-      </c>
-      <c r="V5" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="W5" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="X5" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y5" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="Z5" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="AA5" s="22" t="s">
-        <v>100</v>
-      </c>
-      <c r="AB5" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="AC5" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="AD5" s="22" t="s">
-        <v>103</v>
-      </c>
-      <c r="AE5" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="AF5" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="AG5" s="24" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="6" spans="2:33" x14ac:dyDescent="0.45">
       <c r="B6" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>4</v>
@@ -1562,92 +1632,112 @@
         <v>3</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F6" s="9">
-        <v>45930</v>
-      </c>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
+        <v>45838</v>
+      </c>
+      <c r="G6" s="49">
+        <v>48821746</v>
+      </c>
+      <c r="H6" s="49">
+        <v>3969841</v>
+      </c>
+      <c r="I6" s="49">
+        <v>820000</v>
+      </c>
+      <c r="J6" s="49">
+        <v>366900</v>
+      </c>
+      <c r="K6" s="49">
+        <v>356406000000</v>
+      </c>
+      <c r="L6" s="11">
+        <v>0.308</v>
+      </c>
       <c r="M6" s="12">
-        <v>1.2800000000000001E-2</v>
+        <v>0.14099999999999999</v>
       </c>
       <c r="N6" s="12">
-        <v>0.26550000000000001</v>
-      </c>
-      <c r="O6" s="45">
-        <v>9.2999999999999999E-2</v>
-      </c>
-      <c r="P6" s="46">
-        <v>1.6E-2</v>
-      </c>
-      <c r="Q6" s="47">
-        <v>12.49</v>
-      </c>
-      <c r="R6" s="45">
-        <v>0.44519999999999998</v>
-      </c>
-      <c r="S6" s="47">
-        <v>11.7</v>
-      </c>
-      <c r="T6" s="47">
-        <v>11.7</v>
-      </c>
-      <c r="U6" s="47">
-        <v>0.99</v>
-      </c>
-      <c r="V6" s="47">
-        <v>0.94</v>
-      </c>
-      <c r="W6" s="48">
-        <v>0.308</v>
-      </c>
-      <c r="X6" s="6">
-        <f>W6/U6</f>
-        <v>0.31111111111111112</v>
+        <v>1.55E-2</v>
+      </c>
+      <c r="O6" s="12">
+        <v>0.25269999999999998</v>
+      </c>
+      <c r="P6" s="36">
+        <f t="shared" ref="P6:P8" si="0">J6/H6</f>
+        <v>9.2421837549665084E-2</v>
+      </c>
+      <c r="Q6" s="37">
+        <f>I6/G6</f>
+        <v>1.679579423480676E-2</v>
+      </c>
+      <c r="R6" s="38">
+        <f>G6/H6</f>
+        <v>12.298161563649527</v>
+      </c>
+      <c r="S6" s="36">
+        <f>J6/I6</f>
+        <v>0.44743902439024391</v>
+      </c>
+      <c r="T6" s="38">
+        <f t="shared" ref="T6:T11" si="1">H6/(K6/1000000)*$AF6</f>
+        <v>11.138535827118512</v>
+      </c>
+      <c r="U6" s="38">
+        <f t="shared" ref="U6:U11" si="2">J6/(K6/1000000)*$AF6</f>
+        <v>1.0294439487550715</v>
+      </c>
+      <c r="V6" s="6">
+        <f>L6/U6</f>
+        <v>0.29919064595257561</v>
+      </c>
+      <c r="W6" s="7">
+        <f>(P6-g)/(k-g)</f>
+        <v>0.90527296937081347</v>
+      </c>
+      <c r="X6" s="7">
+        <f>T6*W6</f>
+        <v>10.083415402658765</v>
       </c>
       <c r="Y6" s="7">
-        <f>(O6-g)/(k-g)</f>
-        <v>0.91249999999999998</v>
+        <f>PV(Target_return,Holding_Period,-L6,-X6)</f>
+        <v>5.2103294940404279</v>
       </c>
       <c r="Z6" s="7">
-        <f>T6*Y6</f>
-        <v>10.67625</v>
+        <f>PV(Entry_yield,Holding_Period,-L6,-X6)</f>
+        <v>6.4723886829985986</v>
       </c>
       <c r="AA6" s="7">
-        <f>PV(Target_return,Holding_Period,-W6,-Z6)</f>
-        <v>5.4835251610179547</v>
+        <f>PV(Benchmark_yield,Holding_Period,-L6,-X6)</f>
+        <v>7.9704745497303149</v>
       </c>
       <c r="AB6" s="7">
-        <f>PV(Entry_yield,Holding_Period,-W6,-Z6)</f>
-        <v>6.8148202193689871</v>
-      </c>
-      <c r="AC6" s="7">
-        <f>PV(Benchmark_yield,Holding_Period,-W6,-Z6)</f>
-        <v>8.3953949087133903</v>
-      </c>
-      <c r="AD6" s="7">
-        <f>PV(Base_Cost_of_Equity,Holding_Period,-W6,-Z6)</f>
-        <v>9.4588096710841096</v>
-      </c>
-      <c r="AE6" s="13">
+        <f>PV(Base_Cost_of_Equity,Holding_Period,-L6,-X6)</f>
+        <v>8.9782562888960111</v>
+      </c>
+      <c r="AC6" s="13">
         <v>7.43</v>
       </c>
-      <c r="AF6" s="7" t="s">
+      <c r="AD6" s="7" t="s">
         <v>3</v>
       </c>
+      <c r="AE6" s="7" t="str">
+        <f>AD6&amp;D6</f>
+        <v>CNYCNY</v>
+      </c>
+      <c r="AF6" s="7">
+        <f>IFERROR(VLOOKUP(AE6,Assumptions!B$12:C$13,2),1)</f>
+        <v>1</v>
+      </c>
       <c r="AG6" s="5">
-        <f>W6/AE6</f>
+        <f>L6/AC6</f>
         <v>4.1453566621803502E-2</v>
       </c>
     </row>
     <row r="7" spans="2:33" x14ac:dyDescent="0.45">
       <c r="B7" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>5</v>
@@ -1656,92 +1746,112 @@
         <v>3</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F7" s="9">
-        <v>45930</v>
-      </c>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
+        <v>45838</v>
+      </c>
+      <c r="G7" s="49">
+        <v>40571149</v>
+      </c>
+      <c r="H7" s="49">
+        <v>3322127</v>
+      </c>
+      <c r="I7" s="49">
+        <v>728570</v>
+      </c>
+      <c r="J7" s="49">
+        <v>335577</v>
+      </c>
+      <c r="K7" s="49">
+        <v>250011000000</v>
+      </c>
+      <c r="L7" s="11">
+        <v>0.38700000000000001</v>
+      </c>
       <c r="M7" s="12">
-        <v>1.3599999999999999E-2</v>
+        <v>0.14480000000000001</v>
       </c>
       <c r="N7" s="12">
-        <v>0.25530000000000003</v>
-      </c>
-      <c r="O7" s="45">
-        <v>0.1032</v>
-      </c>
-      <c r="P7" s="46">
-        <v>1.7399999999999999E-2</v>
-      </c>
-      <c r="Q7" s="47">
-        <v>12.86</v>
-      </c>
-      <c r="R7" s="45">
-        <v>0.4612</v>
-      </c>
-      <c r="S7" s="47">
-        <v>13.5</v>
-      </c>
-      <c r="T7" s="47">
-        <v>13.5</v>
-      </c>
-      <c r="U7" s="47">
-        <v>1.3</v>
-      </c>
-      <c r="V7" s="47">
-        <v>1.29</v>
-      </c>
-      <c r="W7" s="48">
-        <v>0.38700000000000001</v>
-      </c>
-      <c r="X7" s="6">
-        <f t="shared" ref="X7:X11" si="0">W7/U7</f>
-        <v>0.2976923076923077</v>
+        <v>1.5100000000000001E-2</v>
+      </c>
+      <c r="O7" s="12">
+        <v>0.29580000000000001</v>
+      </c>
+      <c r="P7" s="36">
+        <f t="shared" si="0"/>
+        <v>0.10101269457790145</v>
+      </c>
+      <c r="Q7" s="37">
+        <f t="shared" ref="Q7:Q12" si="3">I7/G7</f>
+        <v>1.7957835012264504E-2</v>
+      </c>
+      <c r="R7" s="38">
+        <f t="shared" ref="R7:R12" si="4">G7/H7</f>
+        <v>12.212401572847757</v>
+      </c>
+      <c r="S7" s="36">
+        <f t="shared" ref="S7:S12" si="5">J7/I7</f>
+        <v>0.4605967854838931</v>
+      </c>
+      <c r="T7" s="38">
+        <f t="shared" si="1"/>
+        <v>13.28792333137342</v>
+      </c>
+      <c r="U7" s="38">
+        <f t="shared" si="2"/>
+        <v>1.3422489410465939</v>
+      </c>
+      <c r="V7" s="6">
+        <f>L7/U7</f>
+        <v>0.28832207511241836</v>
+      </c>
+      <c r="W7" s="7">
+        <f>(P7-g)/(k-g)</f>
+        <v>1.012658682223768</v>
+      </c>
+      <c r="X7" s="7">
+        <f>T7*W7</f>
+        <v>13.45613093023907</v>
       </c>
       <c r="Y7" s="7">
-        <f>(O7-g)/(k-g)</f>
-        <v>1.04</v>
+        <f>PV(Target_return,Holding_Period,-L7,-X7)</f>
+        <v>6.9091345554564931</v>
       </c>
       <c r="Z7" s="7">
-        <f>T7*Y7</f>
-        <v>14.040000000000001</v>
+        <f>PV(Entry_yield,Holding_Period,-L7,-X7)</f>
+        <v>8.5867439277312272</v>
       </c>
       <c r="AA7" s="7">
-        <f>PV(Target_return,Holding_Period,-W7,-Z7)</f>
-        <v>7.1781986429039275</v>
+        <f>PV(Benchmark_yield,Holding_Period,-L7,-X7)</f>
+        <v>10.578499103755053</v>
       </c>
       <c r="AB7" s="7">
-        <f>PV(Entry_yield,Holding_Period,-W7,-Z7)</f>
-        <v>8.9239968200119097</v>
-      </c>
-      <c r="AC7" s="7">
-        <f>PV(Benchmark_yield,Holding_Period,-W7,-Z7)</f>
-        <v>10.996993327666086</v>
-      </c>
-      <c r="AD7" s="7">
-        <f>PV(Base_Cost_of_Equity,Holding_Period,-W7,-Z7)</f>
-        <v>12.391852469176545</v>
-      </c>
-      <c r="AE7" s="13">
+        <f>PV(Base_Cost_of_Equity,Holding_Period,-L7,-X7)</f>
+        <v>11.918566568712924</v>
+      </c>
+      <c r="AC7" s="13">
         <v>8.91</v>
       </c>
-      <c r="AF7" s="7" t="s">
+      <c r="AD7" s="7" t="s">
         <v>3</v>
       </c>
+      <c r="AE7" s="7" t="str">
+        <f t="shared" ref="AE7:AE12" si="6">AD7&amp;D7</f>
+        <v>CNYCNY</v>
+      </c>
+      <c r="AF7" s="7">
+        <f>IFERROR(VLOOKUP(AE7,Assumptions!B$12:C$13,2),1)</f>
+        <v>1</v>
+      </c>
       <c r="AG7" s="5">
-        <f>W7/AE7</f>
+        <f>L7/AC7</f>
         <v>4.3434343434343436E-2</v>
       </c>
     </row>
     <row r="8" spans="2:33" x14ac:dyDescent="0.45">
       <c r="B8" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>6</v>
@@ -1750,92 +1860,112 @@
         <v>3</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F8" s="9">
-        <v>45930</v>
-      </c>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
+        <v>45838</v>
+      </c>
+      <c r="G8" s="49">
+        <v>43238135</v>
+      </c>
+      <c r="H8" s="49">
+        <v>3090808</v>
+      </c>
+      <c r="I8" s="49">
+        <v>711416</v>
+      </c>
+      <c r="J8" s="49">
+        <v>282671</v>
+      </c>
+      <c r="K8" s="49">
+        <v>349983000000</v>
+      </c>
+      <c r="L8" s="11">
+        <v>0.23799999999999999</v>
+      </c>
       <c r="M8" s="12">
-        <v>1.2999999999999999E-2</v>
+        <v>0.1163</v>
       </c>
       <c r="N8" s="12">
-        <v>0.29139999999999999</v>
-      </c>
-      <c r="O8" s="45">
-        <v>0.1047</v>
-      </c>
-      <c r="P8" s="46">
-        <v>1.5900000000000001E-2</v>
-      </c>
-      <c r="Q8" s="47">
-        <v>16.38</v>
-      </c>
-      <c r="R8" s="45">
-        <v>0.40100000000000002</v>
-      </c>
-      <c r="S8" s="47">
-        <v>8.59</v>
-      </c>
-      <c r="T8" s="47">
-        <v>8.59</v>
-      </c>
-      <c r="U8" s="47">
-        <v>0.78</v>
-      </c>
-      <c r="V8" s="47">
-        <v>0.7</v>
-      </c>
-      <c r="W8" s="48">
-        <v>0.23799999999999999</v>
-      </c>
-      <c r="X8" s="6">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="O8" s="12">
+        <v>0.34399999999999997</v>
+      </c>
+      <c r="P8" s="36">
         <f t="shared" si="0"/>
-        <v>0.3051282051282051</v>
+        <v>9.1455373481626814E-2</v>
+      </c>
+      <c r="Q8" s="37">
+        <f t="shared" si="3"/>
+        <v>1.6453438613853257E-2</v>
+      </c>
+      <c r="R8" s="38">
+        <f t="shared" si="4"/>
+        <v>13.989265913638116</v>
+      </c>
+      <c r="S8" s="36">
+        <f t="shared" si="5"/>
+        <v>0.39733573605316719</v>
+      </c>
+      <c r="T8" s="38">
+        <f t="shared" si="1"/>
+        <v>8.831308949291822</v>
+      </c>
+      <c r="U8" s="38">
+        <f t="shared" si="2"/>
+        <v>0.80767065828911688</v>
+      </c>
+      <c r="V8" s="6">
+        <f>L8/U8</f>
+        <v>0.2946745651304874</v>
+      </c>
+      <c r="W8" s="7">
+        <f>(P8-g)/(k-g)</f>
+        <v>0.89319216852033512</v>
+      </c>
+      <c r="X8" s="7">
+        <f>T8*W8</f>
+        <v>7.8880559912910044</v>
       </c>
       <c r="Y8" s="7">
-        <f>(O8-g)/(k-g)</f>
-        <v>1.0587499999999999</v>
+        <f>PV(Target_return,Holding_Period,-L8,-X8)</f>
+        <v>4.0705535190271149</v>
       </c>
       <c r="Z8" s="7">
-        <f>T8*Y8</f>
-        <v>9.0946624999999983</v>
+        <f>PV(Entry_yield,Holding_Period,-L8,-X8)</f>
+        <v>5.0570307683545934</v>
       </c>
       <c r="AA8" s="7">
-        <f>PV(Target_return,Holding_Period,-W8,-Z8)</f>
-        <v>4.6265933847916285</v>
+        <f>PV(Benchmark_yield,Holding_Period,-L8,-X8)</f>
+        <v>6.2280456564139071</v>
       </c>
       <c r="AB8" s="7">
-        <f>PV(Entry_yield,Holding_Period,-W8,-Z8)</f>
-        <v>5.7539875964897522</v>
-      </c>
-      <c r="AC8" s="7">
-        <f>PV(Benchmark_yield,Holding_Period,-W8,-Z8)</f>
-        <v>7.0928934118103841</v>
-      </c>
-      <c r="AD8" s="7">
-        <f>PV(Base_Cost_of_Equity,Holding_Period,-W8,-Z8)</f>
-        <v>7.9939041555159687</v>
-      </c>
-      <c r="AE8" s="13">
+        <f>PV(Base_Cost_of_Equity,Holding_Period,-L8,-X8)</f>
+        <v>7.0158255458485144</v>
+      </c>
+      <c r="AC8" s="13">
         <v>6.96</v>
       </c>
-      <c r="AF8" s="7" t="s">
+      <c r="AD8" s="7" t="s">
         <v>3</v>
       </c>
+      <c r="AE8" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>CNYCNY</v>
+      </c>
+      <c r="AF8" s="7">
+        <f>IFERROR(VLOOKUP(AE8,Assumptions!B$12:C$13,2),1)</f>
+        <v>1</v>
+      </c>
       <c r="AG8" s="5">
-        <f>W8/AE8</f>
+        <f>L8/AC8</f>
         <v>3.4195402298850576E-2</v>
       </c>
     </row>
     <row r="9" spans="2:33" x14ac:dyDescent="0.45">
       <c r="B9" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>7</v>
@@ -1844,92 +1974,112 @@
         <v>3</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F9" s="9">
-        <v>45930</v>
-      </c>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
+        <v>45838</v>
+      </c>
+      <c r="G9" s="49">
+        <v>35061299</v>
+      </c>
+      <c r="H9" s="49">
+        <v>2816231</v>
+      </c>
+      <c r="I9" s="49">
+        <v>632771</v>
+      </c>
+      <c r="J9" s="49">
+        <v>252700</v>
+      </c>
+      <c r="K9" s="49">
+        <v>294388000000</v>
+      </c>
+      <c r="L9" s="11">
+        <v>0.22900000000000001</v>
+      </c>
       <c r="M9" s="12">
-        <v>1.26E-2</v>
+        <v>0.122</v>
       </c>
       <c r="N9" s="12">
-        <v>0.27</v>
-      </c>
-      <c r="O9" s="45">
-        <v>0.09</v>
-      </c>
-      <c r="P9" s="46">
-        <v>1.6E-2</v>
-      </c>
-      <c r="Q9" s="47">
-        <v>12.5</v>
-      </c>
-      <c r="R9" s="45">
-        <v>0.38500000000000001</v>
-      </c>
-      <c r="S9" s="47">
-        <v>9.1199999999999992</v>
-      </c>
-      <c r="T9" s="47">
-        <v>9.1199999999999992</v>
-      </c>
-      <c r="U9" s="47">
-        <v>0.75</v>
-      </c>
-      <c r="V9" s="47">
-        <v>0.72</v>
-      </c>
-      <c r="W9" s="48">
-        <v>0.22900000000000001</v>
-      </c>
-      <c r="X9" s="6">
-        <f t="shared" si="0"/>
-        <v>0.30533333333333335</v>
+        <v>1.4E-2</v>
+      </c>
+      <c r="O9" s="12">
+        <v>0.28770000000000001</v>
+      </c>
+      <c r="P9" s="36">
+        <f>J9/H9</f>
+        <v>8.9729855256901872E-2</v>
+      </c>
+      <c r="Q9" s="37">
+        <f t="shared" si="3"/>
+        <v>1.8047562926861323E-2</v>
+      </c>
+      <c r="R9" s="38">
+        <f t="shared" si="4"/>
+        <v>12.449724117091247</v>
+      </c>
+      <c r="S9" s="36">
+        <f t="shared" si="5"/>
+        <v>0.39935458483400788</v>
+      </c>
+      <c r="T9" s="38">
+        <f t="shared" si="1"/>
+        <v>9.5663919724988791</v>
+      </c>
+      <c r="U9" s="38">
+        <f t="shared" si="2"/>
+        <v>0.85839096702311235</v>
+      </c>
+      <c r="V9" s="6">
+        <f>L9/U9</f>
+        <v>0.26677820340324498</v>
+      </c>
+      <c r="W9" s="7">
+        <f>(P9-g)/(k-g)</f>
+        <v>0.87162319071127337</v>
+      </c>
+      <c r="X9" s="7">
+        <f>T9*W9</f>
+        <v>8.3382890946641854</v>
       </c>
       <c r="Y9" s="7">
-        <f>(O9-g)/(k-g)</f>
-        <v>0.87499999999999989</v>
+        <f>PV(Target_return,Holding_Period,-L9,-X9)</f>
+        <v>4.2615655476408243</v>
       </c>
       <c r="Z9" s="7">
-        <f>T9*Y9</f>
-        <v>7.9799999999999986</v>
+        <f>PV(Entry_yield,Holding_Period,-L9,-X9)</f>
+        <v>5.2981571752107932</v>
       </c>
       <c r="AA9" s="7">
-        <f>PV(Target_return,Holding_Period,-W9,-Z9)</f>
-        <v>4.0964553657679277</v>
+        <f>PV(Benchmark_yield,Holding_Period,-L9,-X9)</f>
+        <v>6.5290414844024953</v>
       </c>
       <c r="AB9" s="7">
-        <f>PV(Entry_yield,Holding_Period,-W9,-Z9)</f>
-        <v>5.0912031855130682</v>
-      </c>
-      <c r="AC9" s="7">
-        <f>PV(Benchmark_yield,Holding_Period,-W9,-Z9)</f>
-        <v>6.2722340520980744</v>
-      </c>
-      <c r="AD9" s="7">
-        <f>PV(Base_Cost_of_Equity,Holding_Period,-W9,-Z9)</f>
-        <v>7.0668442393416715</v>
-      </c>
-      <c r="AE9" s="13">
+        <f>PV(Base_Cost_of_Equity,Holding_Period,-L9,-X9)</f>
+        <v>7.3572743812635029</v>
+      </c>
+      <c r="AC9" s="13">
         <v>5.38</v>
       </c>
-      <c r="AF9" s="7" t="s">
+      <c r="AD9" s="7" t="s">
         <v>3</v>
       </c>
+      <c r="AE9" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>CNYCNY</v>
+      </c>
+      <c r="AF9" s="7">
+        <f>IFERROR(VLOOKUP(AE9,Assumptions!B$12:C$13,2),1)</f>
+        <v>1</v>
+      </c>
       <c r="AG9" s="5">
-        <f>W9/AE9</f>
+        <f>L9/AC9</f>
         <v>4.2565055762081784E-2</v>
       </c>
     </row>
     <row r="10" spans="2:33" x14ac:dyDescent="0.45">
       <c r="B10" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>8</v>
@@ -1938,92 +2088,112 @@
         <v>3</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F10" s="9">
-        <v>45930</v>
-      </c>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12"/>
+        <v>45838</v>
+      </c>
+      <c r="G10" s="49">
+        <v>10510731</v>
+      </c>
+      <c r="H10" s="49">
+        <v>766132</v>
+      </c>
+      <c r="I10" s="49">
+        <v>212226</v>
+      </c>
+      <c r="J10" s="49">
+        <v>77205</v>
+      </c>
+      <c r="K10" s="49">
+        <v>20774000000</v>
+      </c>
+      <c r="L10" s="50">
+        <v>1.06</v>
+      </c>
       <c r="M10" s="12">
-        <v>1.7000000000000001E-2</v>
+        <v>9.7500000000000003E-2</v>
       </c>
       <c r="N10" s="12">
-        <v>0.3</v>
-      </c>
-      <c r="O10" s="45">
-        <v>8.7400000000000005E-2</v>
-      </c>
-      <c r="P10" s="46">
-        <v>1.5599999999999999E-2</v>
-      </c>
-      <c r="Q10" s="47">
-        <v>12.64</v>
-      </c>
-      <c r="R10" s="45">
+        <v>1.72E-2</v>
+      </c>
+      <c r="O10" s="12">
         <v>0.47599999999999998</v>
       </c>
-      <c r="S10" s="47">
-        <v>36.89</v>
-      </c>
-      <c r="T10" s="47">
-        <v>36.89</v>
-      </c>
-      <c r="U10" s="47">
-        <v>3.21</v>
-      </c>
-      <c r="V10" s="47">
-        <v>3.21</v>
-      </c>
-      <c r="W10" s="49">
-        <v>1.06</v>
-      </c>
-      <c r="X10" s="6">
-        <f t="shared" si="0"/>
-        <v>0.33021806853582558</v>
+      <c r="P10" s="36">
+        <f t="shared" ref="P10:P12" si="7">J10/H10</f>
+        <v>0.10077245174460799</v>
+      </c>
+      <c r="Q10" s="37">
+        <f t="shared" si="3"/>
+        <v>2.0191364425557079E-2</v>
+      </c>
+      <c r="R10" s="38">
+        <f t="shared" si="4"/>
+        <v>13.719216792928634</v>
+      </c>
+      <c r="S10" s="36">
+        <f t="shared" si="5"/>
+        <v>0.36378671793276979</v>
+      </c>
+      <c r="T10" s="38">
+        <f t="shared" si="1"/>
+        <v>36.879368441320885</v>
+      </c>
+      <c r="U10" s="38">
+        <f t="shared" si="2"/>
+        <v>3.716424376624627</v>
+      </c>
+      <c r="V10" s="6">
+        <f>L10/U10</f>
+        <v>0.28522038728061655</v>
+      </c>
+      <c r="W10" s="7">
+        <f>(P10-g)/(k-g)</f>
+        <v>1.0096556468075997</v>
+      </c>
+      <c r="X10" s="7">
+        <f>T10*W10</f>
+        <v>37.235462597477614</v>
       </c>
       <c r="Y10" s="7">
-        <f>(O10-g)/(k-g)</f>
-        <v>0.84250000000000003</v>
+        <f>PV(Target_return,Holding_Period,-L10,-X10)</f>
+        <v>19.098842024353051</v>
       </c>
       <c r="Z10" s="7">
-        <f>T10*Y10</f>
-        <v>31.079825000000003</v>
+        <f>PV(Entry_yield,Holding_Period,-L10,-X10)</f>
+        <v>23.738092615861252</v>
       </c>
       <c r="AA10" s="7">
-        <f>PV(Target_return,Holding_Period,-W10,-Z10)</f>
-        <v>16.262142670676731</v>
+        <f>PV(Benchmark_yield,Holding_Period,-L10,-X10)</f>
+        <v>29.246264118951007</v>
       </c>
       <c r="AB10" s="7">
-        <f>PV(Entry_yield,Holding_Period,-W10,-Z10)</f>
-        <v>20.182489671469853</v>
-      </c>
-      <c r="AC10" s="7">
-        <f>PV(Benchmark_yield,Holding_Period,-W10,-Z10)</f>
-        <v>24.834146895326256</v>
-      </c>
-      <c r="AD10" s="7">
-        <f>PV(Base_Cost_of_Equity,Holding_Period,-W10,-Z10)</f>
-        <v>27.962510785925137</v>
-      </c>
-      <c r="AE10" s="13">
+        <f>PV(Base_Cost_of_Equity,Holding_Period,-L10,-X10)</f>
+        <v>32.952287833787608</v>
+      </c>
+      <c r="AC10" s="13">
         <v>20.09</v>
       </c>
-      <c r="AF10" s="7" t="s">
+      <c r="AD10" s="7" t="s">
         <v>3</v>
       </c>
+      <c r="AE10" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>CNYCNY</v>
+      </c>
+      <c r="AF10" s="7">
+        <f>IFERROR(VLOOKUP(AE10,Assumptions!B$12:C$13,2),1)</f>
+        <v>1</v>
+      </c>
       <c r="AG10" s="5">
-        <f>W10/AE10</f>
+        <f>L10/AC10</f>
         <v>5.2762568442010951E-2</v>
       </c>
     </row>
     <row r="11" spans="2:33" x14ac:dyDescent="0.45">
       <c r="B11" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>9</v>
@@ -2032,107 +2202,235 @@
         <v>3</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F11" s="9">
-        <v>45930</v>
-      </c>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
+        <v>45838</v>
+      </c>
+      <c r="G11" s="49">
+        <v>17084910</v>
+      </c>
+      <c r="H11" s="49">
+        <v>1023006</v>
+      </c>
+      <c r="I11" s="49">
+        <v>349133</v>
+      </c>
+      <c r="J11" s="49">
+        <v>86479</v>
+      </c>
+      <c r="K11" s="49">
+        <v>99161000000</v>
+      </c>
+      <c r="L11" s="50">
+        <v>0.24</v>
+      </c>
       <c r="M11" s="12">
-        <v>1.4E-2</v>
+        <v>9.4799999999999995E-2</v>
       </c>
       <c r="N11" s="12">
-        <v>0.32</v>
-      </c>
-      <c r="O11" s="45">
-        <v>7.9600000000000004E-2</v>
-      </c>
-      <c r="P11" s="46">
-        <v>1.9400000000000001E-2</v>
-      </c>
-      <c r="Q11" s="47">
-        <v>16.3</v>
-      </c>
-      <c r="R11" s="45">
+        <v>1.8700000000000001E-2</v>
+      </c>
+      <c r="O11" s="12">
         <v>0.252</v>
       </c>
-      <c r="S11" s="47">
-        <v>8.44</v>
-      </c>
-      <c r="T11" s="47">
-        <v>8.44</v>
-      </c>
-      <c r="U11" s="47">
-        <v>0.76</v>
-      </c>
-      <c r="V11" s="47">
-        <v>0.76</v>
-      </c>
-      <c r="W11" s="49">
-        <v>0.24</v>
-      </c>
-      <c r="X11" s="6">
-        <f t="shared" si="0"/>
-        <v>0.31578947368421051</v>
+      <c r="P11" s="36">
+        <f t="shared" si="7"/>
+        <v>8.4534206055487462E-2</v>
+      </c>
+      <c r="Q11" s="37">
+        <f t="shared" si="3"/>
+        <v>2.0435167642088838E-2</v>
+      </c>
+      <c r="R11" s="38">
+        <f t="shared" si="4"/>
+        <v>16.7006938375728</v>
+      </c>
+      <c r="S11" s="36">
+        <f t="shared" si="5"/>
+        <v>0.24769643660152435</v>
+      </c>
+      <c r="T11" s="38">
+        <f t="shared" si="1"/>
+        <v>10.316616411694113</v>
+      </c>
+      <c r="U11" s="38">
+        <f t="shared" si="2"/>
+        <v>0.87210697754157385</v>
+      </c>
+      <c r="V11" s="6">
+        <f>L11/U11</f>
+        <v>0.27519559661883231</v>
+      </c>
+      <c r="W11" s="7">
+        <f>(P11-g)/(k-g)</f>
+        <v>0.80667757569359322</v>
+      </c>
+      <c r="X11" s="7">
+        <f>T11*W11</f>
+        <v>8.3221831163461442</v>
       </c>
       <c r="Y11" s="7">
-        <f>(O11-g)/(k-g)</f>
-        <v>0.745</v>
+        <f>PV(Target_return,Holding_Period,-L11,-X11)</f>
+        <v>4.2742718051540534</v>
       </c>
       <c r="Z11" s="7">
-        <f>T11*Y11</f>
-        <v>6.2877999999999998</v>
+        <f>PV(Entry_yield,Holding_Period,-L11,-X11)</f>
+        <v>5.3119981264614875</v>
       </c>
       <c r="AA11" s="7">
-        <f>PV(Target_return,Holding_Period,-W11,-Z11)</f>
-        <v>3.3367680649023743</v>
+        <f>PV(Benchmark_yield,Holding_Period,-L11,-X11)</f>
+        <v>6.5440359914386921</v>
       </c>
       <c r="AB11" s="7">
-        <f>PV(Entry_yield,Holding_Period,-W11,-Z11)</f>
-        <v>4.136903185611728</v>
-      </c>
-      <c r="AC11" s="7">
-        <f>PV(Benchmark_yield,Holding_Period,-W11,-Z11)</f>
-        <v>5.0858707494237514</v>
-      </c>
-      <c r="AD11" s="7">
-        <f>PV(Base_Cost_of_Equity,Holding_Period,-W11,-Z11)</f>
-        <v>5.7238783153986832</v>
-      </c>
-      <c r="AE11" s="13">
+        <f>PV(Base_Cost_of_Equity,Holding_Period,-L11,-X11)</f>
+        <v>7.3729549577050042</v>
+      </c>
+      <c r="AC11" s="13">
         <v>5.17</v>
       </c>
-      <c r="AF11" s="7" t="s">
+      <c r="AD11" s="7" t="s">
         <v>3</v>
       </c>
+      <c r="AE11" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>CNYCNY</v>
+      </c>
+      <c r="AF11" s="7">
+        <f>IFERROR(VLOOKUP(AE11,Assumptions!B$12:C$13,2),1)</f>
+        <v>1</v>
+      </c>
       <c r="AG11" s="5">
-        <f>W11/AE11</f>
+        <f>L11/AC11</f>
         <v>4.6421663442940041E-2</v>
       </c>
     </row>
     <row r="12" spans="2:33" x14ac:dyDescent="0.45">
-      <c r="X12" s="19"/>
-      <c r="AA12" s="18"/>
-      <c r="AB12" s="18"/>
-      <c r="AC12" s="18"/>
-      <c r="AD12" s="18"/>
+      <c r="B12" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" s="9">
+        <v>45838</v>
+      </c>
+      <c r="G12" s="49">
+        <v>3017048</v>
+      </c>
+      <c r="H12" s="49">
+        <v>154295</v>
+      </c>
+      <c r="I12" s="49">
+        <v>51910</v>
+      </c>
+      <c r="J12" s="49">
+        <v>23730</v>
+      </c>
+      <c r="K12" s="49">
+        <v>17918000000</v>
+      </c>
+      <c r="L12" s="50">
+        <f>0.780688+0.779073+0.777313+2.791007</f>
+        <v>5.1280809999999999</v>
+      </c>
+      <c r="M12" s="12">
+        <v>0.14899999999999999</v>
+      </c>
+      <c r="N12" s="12">
+        <v>1.4500000000000001E-2</v>
+      </c>
+      <c r="O12" s="12">
+        <v>0.52300000000000002</v>
+      </c>
+      <c r="P12" s="36">
+        <f t="shared" si="7"/>
+        <v>0.15379629929680158</v>
+      </c>
+      <c r="Q12" s="37">
+        <f t="shared" si="3"/>
+        <v>1.7205559871768694E-2</v>
+      </c>
+      <c r="R12" s="38">
+        <f t="shared" si="4"/>
+        <v>19.553763893839722</v>
+      </c>
+      <c r="S12" s="36">
+        <f t="shared" si="5"/>
+        <v>0.45713735311115394</v>
+      </c>
+      <c r="T12" s="38">
+        <f>H12/(K12/1000000)*$AF12</f>
+        <v>67.167150351601748</v>
+      </c>
+      <c r="U12" s="38">
+        <f>J12/(K12/1000000)*$AF12</f>
+        <v>10.330059158388213</v>
+      </c>
+      <c r="V12" s="6">
+        <f>L12/U12</f>
+        <v>0.49642319771575522</v>
+      </c>
+      <c r="W12" s="7">
+        <f>(P12-g)/(k-g)</f>
+        <v>1.6724537412100198</v>
+      </c>
+      <c r="X12" s="7">
+        <f>T12*W12</f>
+        <v>112.33395189195224</v>
+      </c>
+      <c r="Y12" s="7">
+        <f>PV(Target_return,Holding_Period,-L12,-X12)</f>
+        <v>61.150425207160808</v>
+      </c>
+      <c r="Z12" s="7">
+        <f>PV(Entry_yield,Holding_Period,-L12,-X12)</f>
+        <v>75.675539859823033</v>
+      </c>
+      <c r="AA12" s="7">
+        <f>PV(Benchmark_yield,Holding_Period,-L12,-X12)</f>
+        <v>92.888551757648202</v>
+      </c>
+      <c r="AB12" s="7">
+        <f>PV(Base_Cost_of_Equity,Holding_Period,-L12,-X12)</f>
+        <v>104.45468726004771</v>
+      </c>
+      <c r="AC12" s="13">
+        <v>130</v>
+      </c>
+      <c r="AD12" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="AE12" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>HKDUSD</v>
+      </c>
+      <c r="AF12" s="7">
+        <f>IFERROR(VLOOKUP(AE12,Assumptions!B$12:C$13,2),1)</f>
+        <v>7.8</v>
+      </c>
+      <c r="AG12" s="5">
+        <f>L12/AC12</f>
+        <v>3.9446776923076923E-2</v>
+      </c>
     </row>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="6">
-    <mergeCell ref="S3:X3"/>
-    <mergeCell ref="Y3:Z3"/>
-    <mergeCell ref="AE3:AG3"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="W3:X3"/>
+    <mergeCell ref="AC3:AG3"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="E3:K3"/>
-    <mergeCell ref="L3:R3"/>
+    <mergeCell ref="M3:S3"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="50" orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>